<commit_message>
Adding Exercise 1A Python File.
</commit_message>
<xml_diff>
--- a/pre-week-2/homework1.xlsx
+++ b/pre-week-2/homework1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smayamelgara\Documents\DataAnalytics\pre-week-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F732AA44-5E40-4217-9B34-3CC76FAE07E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E42CB1BD-8791-4DE7-9E31-31C6D79771FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11844" yWindow="1452" windowWidth="10788" windowHeight="8256" activeTab="1" xr2:uid="{B8066DCD-FBC7-4888-9E61-30436CADF69E}"/>
+    <workbookView xWindow="11208" yWindow="768" windowWidth="10788" windowHeight="8256" xr2:uid="{B8066DCD-FBC7-4888-9E61-30436CADF69E}"/>
   </bookViews>
   <sheets>
     <sheet name="Store_Data" sheetId="1" r:id="rId1"/>
@@ -99,9 +99,6 @@
     <t xml:space="preserve">Standard Deviation: </t>
   </si>
   <si>
-    <t xml:space="preserve">Standard Deviation 2: </t>
-  </si>
-  <si>
     <t>A. Overall Average Performance :</t>
   </si>
   <si>
@@ -124,6 +121,29 @@
   </si>
   <si>
     <t xml:space="preserve">Any information on why Store H would be performing higher. For example, Location would be a very important and helpful to understand the data, </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Standard Deviation 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
 </sst>
 </file>
@@ -620,7 +640,7 @@
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B15">
@@ -629,7 +649,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B16">
@@ -638,7 +658,7 @@
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B17">
@@ -647,7 +667,7 @@
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B18">
@@ -656,7 +676,7 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B19">
@@ -666,7 +686,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B21">
         <f>_xlfn.STDEV.S(B2:B8,B10:B13)</f>
@@ -675,6 +695,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -689,34 +710,34 @@
   <sheetData>
     <row r="1" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>